<commit_message>
checking about completeness of the 2010 birth data file
</commit_message>
<xml_diff>
--- a/notebooks/2010_Birth/First Stage 2010/01_missing_values.xlsx
+++ b/notebooks/2010_Birth/First Stage 2010/01_missing_values.xlsx
@@ -8,6 +8,7 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Missing Values" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,7 +18,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -25,16 +26,31 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="00000000"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <sz val="9"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F0F0F0"/>
+        <bgColor rgb="00F0F0F0"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -42,12 +58,35 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00CCCCCC"/>
+      </left>
+      <right style="thin">
+        <color rgb="00CCCCCC"/>
+      </right>
+      <top style="thin">
+        <color rgb="00CCCCCC"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00CCCCCC"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -413,7 +452,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E19"/>
+  <dimension ref="A1:G19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -421,411 +460,611 @@
     <col width="11" customWidth="1" min="3" max="3"/>
     <col width="11" customWidth="1" min="4" max="4"/>
     <col width="15" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Variable</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Missing Count</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Missing %</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Data Type</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Unique Values</t>
         </is>
       </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Non-Missing</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Completion %</t>
+        </is>
+      </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Birth_Weight(grams)</t>
         </is>
       </c>
-      <c r="B2" t="n">
+      <c r="B2" s="3" t="n">
         <v>45303</v>
       </c>
-      <c r="C2" t="n">
+      <c r="C2" s="3" t="n">
         <v>12.4</v>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="D2" s="2" t="inlineStr">
         <is>
           <t>float64</t>
         </is>
       </c>
-      <c r="E2" t="n">
+      <c r="E2" s="3" t="n">
         <v>2275</v>
       </c>
+      <c r="F2" s="3" t="n">
+        <v>318578</v>
+      </c>
+      <c r="G2" s="3" t="n">
+        <v>87.59999999999999</v>
+      </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="2" t="inlineStr">
         <is>
           <t>Race_of_Father</t>
         </is>
       </c>
-      <c r="B3" t="n">
+      <c r="B3" s="3" t="n">
         <v>531</v>
       </c>
-      <c r="C3" t="n">
+      <c r="C3" s="3" t="n">
         <v>0.1</v>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="D3" s="2" t="inlineStr">
         <is>
           <t>str</t>
         </is>
       </c>
-      <c r="E3" t="n">
+      <c r="E3" s="3" t="n">
         <v>12</v>
       </c>
+      <c r="F3" s="3" t="n">
+        <v>363350</v>
+      </c>
+      <c r="G3" s="3" t="n">
+        <v>99.90000000000001</v>
+      </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" s="2" t="inlineStr">
         <is>
           <t>Birth_Order</t>
         </is>
       </c>
-      <c r="B4" t="n">
+      <c r="B4" s="3" t="n">
         <v>16</v>
       </c>
-      <c r="C4" t="n">
-        <v>0</v>
-      </c>
-      <c r="D4" t="inlineStr">
+      <c r="C4" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
         <is>
           <t>str</t>
         </is>
       </c>
-      <c r="E4" t="n">
+      <c r="E4" s="3" t="n">
         <v>9</v>
       </c>
+      <c r="F4" s="3" t="n">
+        <v>363865</v>
+      </c>
+      <c r="G4" s="3" t="n">
+        <v>100</v>
+      </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="A5" s="2" t="inlineStr">
         <is>
           <t>Registered_Year</t>
         </is>
       </c>
-      <c r="B5" t="n">
-        <v>0</v>
-      </c>
-      <c r="C5" t="n">
-        <v>0</v>
-      </c>
-      <c r="D5" t="inlineStr">
+      <c r="B5" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C5" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
         <is>
           <t>int64</t>
         </is>
       </c>
-      <c r="E5" t="n">
+      <c r="E5" s="3" t="n">
         <v>1</v>
       </c>
+      <c r="F5" s="3" t="n">
+        <v>363881</v>
+      </c>
+      <c r="G5" s="3" t="n">
+        <v>100</v>
+      </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
+      <c r="A6" s="2" t="inlineStr">
         <is>
           <t>Registered_Month2.0</t>
         </is>
       </c>
-      <c r="B6" t="n">
-        <v>0</v>
-      </c>
-      <c r="C6" t="n">
-        <v>0</v>
-      </c>
-      <c r="D6" t="inlineStr">
+      <c r="B6" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C6" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
         <is>
           <t>int64</t>
         </is>
       </c>
-      <c r="E6" t="n">
+      <c r="E6" s="3" t="n">
         <v>12</v>
       </c>
+      <c r="F6" s="3" t="n">
+        <v>363881</v>
+      </c>
+      <c r="G6" s="3" t="n">
+        <v>100</v>
+      </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
+      <c r="A7" s="2" t="inlineStr">
         <is>
           <t>Registered_Month</t>
         </is>
       </c>
-      <c r="B7" t="n">
-        <v>0</v>
-      </c>
-      <c r="C7" t="n">
-        <v>0</v>
-      </c>
-      <c r="D7" t="inlineStr">
+      <c r="B7" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C7" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
         <is>
           <t>str</t>
         </is>
       </c>
-      <c r="E7" t="n">
+      <c r="E7" s="3" t="n">
         <v>12</v>
       </c>
+      <c r="F7" s="3" t="n">
+        <v>363881</v>
+      </c>
+      <c r="G7" s="3" t="n">
+        <v>100</v>
+      </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
+      <c r="A8" s="2" t="inlineStr">
         <is>
           <t>Birth_Month.0</t>
         </is>
       </c>
-      <c r="B8" t="n">
-        <v>0</v>
-      </c>
-      <c r="C8" t="n">
-        <v>0</v>
-      </c>
-      <c r="D8" t="inlineStr">
+      <c r="B8" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C8" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
         <is>
           <t>int64</t>
         </is>
       </c>
-      <c r="E8" t="n">
+      <c r="E8" s="3" t="n">
         <v>12</v>
       </c>
+      <c r="F8" s="3" t="n">
+        <v>363881</v>
+      </c>
+      <c r="G8" s="3" t="n">
+        <v>100</v>
+      </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
+      <c r="A9" s="2" t="inlineStr">
         <is>
           <t>Registered_District_2.0</t>
         </is>
       </c>
-      <c r="B9" t="n">
-        <v>0</v>
-      </c>
-      <c r="C9" t="n">
-        <v>0</v>
-      </c>
-      <c r="D9" t="inlineStr">
+      <c r="B9" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C9" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
         <is>
           <t>int64</t>
         </is>
       </c>
-      <c r="E9" t="n">
+      <c r="E9" s="3" t="n">
         <v>25</v>
       </c>
+      <c r="F9" s="3" t="n">
+        <v>363881</v>
+      </c>
+      <c r="G9" s="3" t="n">
+        <v>100</v>
+      </c>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr">
+      <c r="A10" s="2" t="inlineStr">
         <is>
           <t>Registered_District</t>
         </is>
       </c>
-      <c r="B10" t="n">
-        <v>0</v>
-      </c>
-      <c r="C10" t="n">
-        <v>0</v>
-      </c>
-      <c r="D10" t="inlineStr">
+      <c r="B10" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C10" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
         <is>
           <t>str</t>
         </is>
       </c>
-      <c r="E10" t="n">
+      <c r="E10" s="3" t="n">
         <v>25</v>
       </c>
+      <c r="F10" s="3" t="n">
+        <v>363881</v>
+      </c>
+      <c r="G10" s="3" t="n">
+        <v>100</v>
+      </c>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr">
+      <c r="A11" s="2" t="inlineStr">
         <is>
           <t>Birh_Year</t>
         </is>
       </c>
-      <c r="B11" t="n">
-        <v>0</v>
-      </c>
-      <c r="C11" t="n">
-        <v>0</v>
-      </c>
-      <c r="D11" t="inlineStr">
+      <c r="B11" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C11" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
         <is>
           <t>int64</t>
         </is>
       </c>
-      <c r="E11" t="n">
+      <c r="E11" s="3" t="n">
         <v>60</v>
       </c>
+      <c r="F11" s="3" t="n">
+        <v>363881</v>
+      </c>
+      <c r="G11" s="3" t="n">
+        <v>100</v>
+      </c>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr">
+      <c r="A12" s="2" t="inlineStr">
         <is>
           <t>Hospital or Not</t>
         </is>
       </c>
-      <c r="B12" t="n">
-        <v>0</v>
-      </c>
-      <c r="C12" t="n">
-        <v>0</v>
-      </c>
-      <c r="D12" t="inlineStr">
+      <c r="B12" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C12" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
         <is>
           <t>str</t>
         </is>
       </c>
-      <c r="E12" t="n">
+      <c r="E12" s="3" t="n">
         <v>2</v>
       </c>
+      <c r="F12" s="3" t="n">
+        <v>363881</v>
+      </c>
+      <c r="G12" s="3" t="n">
+        <v>100</v>
+      </c>
     </row>
     <row r="13">
-      <c r="A13" t="inlineStr">
+      <c r="A13" s="2" t="inlineStr">
         <is>
           <t>Gender</t>
         </is>
       </c>
-      <c r="B13" t="n">
-        <v>0</v>
-      </c>
-      <c r="C13" t="n">
-        <v>0</v>
-      </c>
-      <c r="D13" t="inlineStr">
+      <c r="B13" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C13" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
         <is>
           <t>str</t>
         </is>
       </c>
-      <c r="E13" t="n">
+      <c r="E13" s="3" t="n">
         <v>2</v>
       </c>
+      <c r="F13" s="3" t="n">
+        <v>363881</v>
+      </c>
+      <c r="G13" s="3" t="n">
+        <v>100</v>
+      </c>
     </row>
     <row r="14">
-      <c r="A14" t="inlineStr">
+      <c r="A14" s="2" t="inlineStr">
         <is>
           <t>Birth_Month</t>
         </is>
       </c>
-      <c r="B14" t="n">
-        <v>0</v>
-      </c>
-      <c r="C14" t="n">
-        <v>0</v>
-      </c>
-      <c r="D14" t="inlineStr">
+      <c r="B14" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C14" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
         <is>
           <t>str</t>
         </is>
       </c>
-      <c r="E14" t="n">
+      <c r="E14" s="3" t="n">
         <v>12</v>
       </c>
+      <c r="F14" s="3" t="n">
+        <v>363881</v>
+      </c>
+      <c r="G14" s="3" t="n">
+        <v>100</v>
+      </c>
     </row>
     <row r="15">
-      <c r="A15" t="inlineStr">
+      <c r="A15" s="2" t="inlineStr">
         <is>
           <t>Multiple_Birth_Status</t>
         </is>
       </c>
-      <c r="B15" t="n">
-        <v>0</v>
-      </c>
-      <c r="C15" t="n">
-        <v>0</v>
-      </c>
-      <c r="D15" t="inlineStr">
+      <c r="B15" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C15" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
         <is>
           <t>str</t>
         </is>
       </c>
-      <c r="E15" t="n">
+      <c r="E15" s="3" t="n">
         <v>2</v>
       </c>
+      <c r="F15" s="3" t="n">
+        <v>363881</v>
+      </c>
+      <c r="G15" s="3" t="n">
+        <v>100</v>
+      </c>
     </row>
     <row r="16">
-      <c r="A16" t="inlineStr">
+      <c r="A16" s="2" t="inlineStr">
         <is>
           <t>Age of Mother</t>
         </is>
       </c>
-      <c r="B16" t="n">
-        <v>0</v>
-      </c>
-      <c r="C16" t="n">
-        <v>0</v>
-      </c>
-      <c r="D16" t="inlineStr">
+      <c r="B16" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C16" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
         <is>
           <t>int64</t>
         </is>
       </c>
-      <c r="E16" t="n">
+      <c r="E16" s="3" t="n">
         <v>43</v>
       </c>
+      <c r="F16" s="3" t="n">
+        <v>363881</v>
+      </c>
+      <c r="G16" s="3" t="n">
+        <v>100</v>
+      </c>
     </row>
     <row r="17">
-      <c r="A17" t="inlineStr">
+      <c r="A17" s="2" t="inlineStr">
         <is>
           <t>Marital_Status</t>
         </is>
       </c>
-      <c r="B17" t="n">
-        <v>0</v>
-      </c>
-      <c r="C17" t="n">
-        <v>0</v>
-      </c>
-      <c r="D17" t="inlineStr">
+      <c r="B17" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C17" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
         <is>
           <t>str</t>
         </is>
       </c>
-      <c r="E17" t="n">
+      <c r="E17" s="3" t="n">
         <v>2</v>
       </c>
+      <c r="F17" s="3" t="n">
+        <v>363881</v>
+      </c>
+      <c r="G17" s="3" t="n">
+        <v>100</v>
+      </c>
     </row>
     <row r="18">
-      <c r="A18" t="inlineStr">
+      <c r="A18" s="2" t="inlineStr">
         <is>
           <t>District_of_Mother</t>
         </is>
       </c>
-      <c r="B18" t="n">
-        <v>0</v>
-      </c>
-      <c r="C18" t="n">
-        <v>0</v>
-      </c>
-      <c r="D18" t="inlineStr">
+      <c r="B18" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C18" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
         <is>
           <t>str</t>
         </is>
       </c>
-      <c r="E18" t="n">
+      <c r="E18" s="3" t="n">
         <v>26</v>
       </c>
+      <c r="F18" s="3" t="n">
+        <v>363881</v>
+      </c>
+      <c r="G18" s="3" t="n">
+        <v>100</v>
+      </c>
     </row>
     <row r="19">
-      <c r="A19" t="inlineStr">
+      <c r="A19" s="2" t="inlineStr">
         <is>
           <t>Race_of_Mother</t>
         </is>
       </c>
-      <c r="B19" t="n">
-        <v>0</v>
-      </c>
-      <c r="C19" t="n">
-        <v>0</v>
-      </c>
-      <c r="D19" t="inlineStr">
+      <c r="B19" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C19" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
         <is>
           <t>str</t>
         </is>
       </c>
-      <c r="E19" t="n">
+      <c r="E19" s="3" t="n">
         <v>12</v>
+      </c>
+      <c r="F19" s="3" t="n">
+        <v>363881</v>
+      </c>
+      <c r="G19" s="3" t="n">
+        <v>100</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="27" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Metric</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Total Rows</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="n">
+        <v>363881</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Total Columns</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="n">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Columns with Missing Data</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Total Missing Values</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="n">
+        <v>45850</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>Overall Missing %</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="n">
+        <v>0.7</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
creating complete data files 2010
</commit_message>
<xml_diff>
--- a/notebooks/2010_Birth/First Stage 2010/01_missing_values.xlsx
+++ b/notebooks/2010_Birth/First Stage 2010/01_missing_values.xlsx
@@ -508,7 +508,7 @@
         </is>
       </c>
       <c r="B2" s="3" t="n">
-        <v>45303</v>
+        <v>45287</v>
       </c>
       <c r="C2" s="3" t="n">
         <v>12.4</v>
@@ -522,7 +522,7 @@
         <v>2275</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>318578</v>
+        <v>318576</v>
       </c>
       <c r="G2" s="3" t="n">
         <v>87.59999999999999</v>
@@ -535,7 +535,7 @@
         </is>
       </c>
       <c r="B3" s="3" t="n">
-        <v>531</v>
+        <v>532</v>
       </c>
       <c r="C3" s="3" t="n">
         <v>0.1</v>
@@ -549,7 +549,7 @@
         <v>12</v>
       </c>
       <c r="F3" s="3" t="n">
-        <v>363350</v>
+        <v>363331</v>
       </c>
       <c r="G3" s="3" t="n">
         <v>99.90000000000001</v>
@@ -562,7 +562,7 @@
         </is>
       </c>
       <c r="B4" s="3" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C4" s="3" t="n">
         <v>0</v>
@@ -576,7 +576,7 @@
         <v>9</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>363865</v>
+        <v>363846</v>
       </c>
       <c r="G4" s="3" t="n">
         <v>100</v>
@@ -589,21 +589,21 @@
         </is>
       </c>
       <c r="B5" s="3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C5" s="3" t="n">
         <v>0</v>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>int64</t>
+          <t>float64</t>
         </is>
       </c>
       <c r="E5" s="3" t="n">
         <v>1</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>363881</v>
+        <v>363862</v>
       </c>
       <c r="G5" s="3" t="n">
         <v>100</v>
@@ -616,21 +616,21 @@
         </is>
       </c>
       <c r="B6" s="3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C6" s="3" t="n">
         <v>0</v>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>int64</t>
+          <t>float64</t>
         </is>
       </c>
       <c r="E6" s="3" t="n">
         <v>12</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>363881</v>
+        <v>363862</v>
       </c>
       <c r="G6" s="3" t="n">
         <v>100</v>
@@ -643,7 +643,7 @@
         </is>
       </c>
       <c r="B7" s="3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C7" s="3" t="n">
         <v>0</v>
@@ -657,7 +657,7 @@
         <v>12</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>363881</v>
+        <v>363862</v>
       </c>
       <c r="G7" s="3" t="n">
         <v>100</v>
@@ -670,21 +670,21 @@
         </is>
       </c>
       <c r="B8" s="3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C8" s="3" t="n">
         <v>0</v>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>int64</t>
+          <t>float64</t>
         </is>
       </c>
       <c r="E8" s="3" t="n">
         <v>12</v>
       </c>
       <c r="F8" s="3" t="n">
-        <v>363881</v>
+        <v>363862</v>
       </c>
       <c r="G8" s="3" t="n">
         <v>100</v>
@@ -697,21 +697,21 @@
         </is>
       </c>
       <c r="B9" s="3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C9" s="3" t="n">
         <v>0</v>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>int64</t>
+          <t>float64</t>
         </is>
       </c>
       <c r="E9" s="3" t="n">
         <v>25</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>363881</v>
+        <v>363862</v>
       </c>
       <c r="G9" s="3" t="n">
         <v>100</v>
@@ -724,7 +724,7 @@
         </is>
       </c>
       <c r="B10" s="3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C10" s="3" t="n">
         <v>0</v>
@@ -738,7 +738,7 @@
         <v>25</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>363881</v>
+        <v>363862</v>
       </c>
       <c r="G10" s="3" t="n">
         <v>100</v>
@@ -751,21 +751,21 @@
         </is>
       </c>
       <c r="B11" s="3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C11" s="3" t="n">
         <v>0</v>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>int64</t>
+          <t>float64</t>
         </is>
       </c>
       <c r="E11" s="3" t="n">
         <v>60</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>363881</v>
+        <v>363862</v>
       </c>
       <c r="G11" s="3" t="n">
         <v>100</v>
@@ -778,7 +778,7 @@
         </is>
       </c>
       <c r="B12" s="3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C12" s="3" t="n">
         <v>0</v>
@@ -792,7 +792,7 @@
         <v>2</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>363881</v>
+        <v>363862</v>
       </c>
       <c r="G12" s="3" t="n">
         <v>100</v>
@@ -805,7 +805,7 @@
         </is>
       </c>
       <c r="B13" s="3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C13" s="3" t="n">
         <v>0</v>
@@ -819,7 +819,7 @@
         <v>2</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>363881</v>
+        <v>363862</v>
       </c>
       <c r="G13" s="3" t="n">
         <v>100</v>
@@ -832,7 +832,7 @@
         </is>
       </c>
       <c r="B14" s="3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C14" s="3" t="n">
         <v>0</v>
@@ -846,7 +846,7 @@
         <v>12</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>363881</v>
+        <v>363862</v>
       </c>
       <c r="G14" s="3" t="n">
         <v>100</v>
@@ -859,7 +859,7 @@
         </is>
       </c>
       <c r="B15" s="3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C15" s="3" t="n">
         <v>0</v>
@@ -873,7 +873,7 @@
         <v>2</v>
       </c>
       <c r="F15" s="3" t="n">
-        <v>363881</v>
+        <v>363862</v>
       </c>
       <c r="G15" s="3" t="n">
         <v>100</v>
@@ -886,21 +886,21 @@
         </is>
       </c>
       <c r="B16" s="3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C16" s="3" t="n">
         <v>0</v>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>int64</t>
+          <t>float64</t>
         </is>
       </c>
       <c r="E16" s="3" t="n">
         <v>43</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>363881</v>
+        <v>363862</v>
       </c>
       <c r="G16" s="3" t="n">
         <v>100</v>
@@ -913,7 +913,7 @@
         </is>
       </c>
       <c r="B17" s="3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C17" s="3" t="n">
         <v>0</v>
@@ -927,7 +927,7 @@
         <v>2</v>
       </c>
       <c r="F17" s="3" t="n">
-        <v>363881</v>
+        <v>363862</v>
       </c>
       <c r="G17" s="3" t="n">
         <v>100</v>
@@ -940,7 +940,7 @@
         </is>
       </c>
       <c r="B18" s="3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C18" s="3" t="n">
         <v>0</v>
@@ -951,10 +951,10 @@
         </is>
       </c>
       <c r="E18" s="3" t="n">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="F18" s="3" t="n">
-        <v>363881</v>
+        <v>363862</v>
       </c>
       <c r="G18" s="3" t="n">
         <v>100</v>
@@ -967,7 +967,7 @@
         </is>
       </c>
       <c r="B19" s="3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C19" s="3" t="n">
         <v>0</v>
@@ -981,7 +981,7 @@
         <v>12</v>
       </c>
       <c r="F19" s="3" t="n">
-        <v>363881</v>
+        <v>363862</v>
       </c>
       <c r="G19" s="3" t="n">
         <v>100</v>
@@ -1024,7 +1024,7 @@
         </is>
       </c>
       <c r="B2" s="3" t="n">
-        <v>363881</v>
+        <v>363863</v>
       </c>
     </row>
     <row r="3">
@@ -1044,7 +1044,7 @@
         </is>
       </c>
       <c r="B4" s="3" t="n">
-        <v>3</v>
+        <v>18</v>
       </c>
     </row>
     <row r="5">
@@ -1054,7 +1054,7 @@
         </is>
       </c>
       <c r="B5" s="3" t="n">
-        <v>45850</v>
+        <v>45851</v>
       </c>
     </row>
     <row r="6">

</xml_diff>